<commit_message>
Allocation units fix (#1265)
* Fixed Copy To all

* Validation added in model for capital_call as validate_unit_prices

* Allocation units update

* Importing Fund units fix

* Removed untested changes

* Removed debug code

* Removed unnecessary Unit calculation complete notification

* Removing the Popup message and checked that decimal is allowing upto 8 digits

* Uploading fund units takes Call Quantity and Distribution Quantity as columns instead of Quantity

* Changed fund_unit to closely match main file

* Copy to all fix test

* Added Useful comments

* Fix for taking the payment date always for fund unit allocation
</commit_message>
<xml_diff>
--- a/public/sample_uploads/fund_units.xlsx
+++ b/public/sample_uploads/fund_units.xlsx
@@ -32,6 +32,7 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -55,6 +56,7 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -79,6 +81,7 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -102,6 +105,7 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -126,6 +130,7 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -143,13 +148,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0">
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -166,13 +172,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -189,13 +196,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -212,13 +220,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -236,13 +245,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0">
+    <comment ref="K1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -264,7 +274,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="20">
   <si>
     <t xml:space="preserve">Fund *</t>
   </si>
@@ -278,7 +288,10 @@
     <t xml:space="preserve">Unit Type *</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantity *</t>
+    <t xml:space="preserve">Call Quantity *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribution Quantity *</t>
   </si>
   <si>
     <t xml:space="preserve">Price *</t>
@@ -331,7 +344,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,11 +394,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
@@ -463,27 +471,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="23" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="23" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -680,7 +688,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
@@ -690,9 +698,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="34.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="34.85"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="1" width="9.06"/>
   </cols>
   <sheetData>
@@ -727,330 +735,337 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="G2" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="H2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="G3" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="H3" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="G4" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="H4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="G5" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="H5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="G6" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G6" s="1" t="n">
+      <c r="H6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="F7" s="1" t="n">
         <v>-5</v>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="G7" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G7" s="1" t="n">
+      <c r="H7" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="H7" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>14</v>
+      <c r="I7" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="F8" s="1" t="n">
         <v>-10</v>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="G8" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G8" s="1" t="n">
+      <c r="H8" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="H8" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>14</v>
+      <c r="I8" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="1" t="n">
+      <c r="F9" s="1" t="n">
         <v>-15</v>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="G9" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G9" s="1" t="n">
+      <c r="H9" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>14</v>
+      <c r="I9" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="1" t="n">
+      <c r="F10" s="1" t="n">
         <v>-20</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="G10" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G10" s="1" t="n">
+      <c r="H10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>14</v>
+      <c r="I10" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="1" t="n">
+      <c r="F11" s="1" t="n">
         <v>-25</v>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="G11" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G11" s="1" t="n">
+      <c r="H11" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>14</v>
+      <c r="I11" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="K11" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I2:I1011" type="list">
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I12:I1011" type="list">
+      <formula1>"Yes,No"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="J2:J11" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Revert "Allocation units fix (#1265)" (#1273)
This reverts commit 22d9533288e66233b3bbbf154d865d7787c6c88e.
</commit_message>
<xml_diff>
--- a/public/sample_uploads/fund_units.xlsx
+++ b/public/sample_uploads/fund_units.xlsx
@@ -32,7 +32,6 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -56,7 +55,6 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -81,7 +79,6 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -105,7 +102,6 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -130,7 +126,6 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -148,14 +143,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="F1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -172,14 +166,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -196,14 +189,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -220,14 +212,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0">
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -245,14 +236,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Author:
 </t>
@@ -274,7 +264,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="19">
   <si>
     <t xml:space="preserve">Fund *</t>
   </si>
@@ -288,10 +278,7 @@
     <t xml:space="preserve">Unit Type *</t>
   </si>
   <si>
-    <t xml:space="preserve">Call Quantity *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distribution Quantity *</t>
+    <t xml:space="preserve">Quantity *</t>
   </si>
   <si>
     <t xml:space="preserve">Price *</t>
@@ -344,7 +331,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -394,6 +381,11 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
@@ -471,27 +463,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="23" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="23" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -688,7 +680,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
@@ -698,9 +690,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="34.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="34.86"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="1" width="9.06"/>
   </cols>
   <sheetData>
@@ -735,337 +727,330 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="G2" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>20</v>
       </c>
+      <c r="F3" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G3" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="I3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>30</v>
       </c>
+      <c r="F4" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G4" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="H4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>40</v>
       </c>
+      <c r="F5" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G5" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="H5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>14</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="D6" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>50</v>
       </c>
+      <c r="F6" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G6" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="H6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>-5</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>-5</v>
-      </c>
-      <c r="G7" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H7" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>19</v>
+      <c r="I7" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="1" t="n">
-        <v>-10</v>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H8" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>19</v>
+      <c r="I8" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>-15</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>-15</v>
-      </c>
-      <c r="G9" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>19</v>
+      <c r="I9" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>-20</v>
-      </c>
-      <c r="G10" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H10" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>19</v>
+      <c r="I10" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>-25</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" s="1" t="n">
-        <v>-25</v>
-      </c>
-      <c r="G11" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H11" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>19</v>
+      <c r="I11" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="1" t="s">
-        <v>16</v>
-      </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I12:I1011" type="list">
-      <formula1>"Yes,No"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="J2:J11" type="list">
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I2:I1011" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>